<commit_message>
Sync pending workspace updates
</commit_message>
<xml_diff>
--- a/docs/PGTA需要统计的指标-20260701.xlsx
+++ b/docs/PGTA需要统计的指标-20260701.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\zhangly\repo\github\yk-hospital-data-review-agent\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4BFD99A-59BB-4F13-ABA3-20159F71701F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C445161B-31CE-4FF5-8101-AF7DB82BD349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{59A484AB-2C44-4318-AC9A-83F77A9CB196}"/>
   </bookViews>
@@ -47,9 +47,6 @@
     <t>计算规则/公式</t>
   </si>
   <si>
-    <t>检测周期数</t>
-  </si>
-  <si>
     <t>检测胚胎数</t>
   </si>
   <si>
@@ -402,6 +399,10 @@
       </rPr>
       <t>（医院可能退而求其次，选择嵌合胚胎去移植）</t>
     </r>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>检测周期数</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -480,7 +481,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -499,6 +500,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -628,7 +635,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -641,6 +648,30 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -650,40 +681,22 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -695,19 +708,31 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1047,22 +1072,23 @@
   <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
+    <col min="3" max="3" width="21.08203125" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="28.6640625" customWidth="1"/>
     <col min="6" max="6" width="99.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="14.5">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="22" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="E1" s="23" t="s">
-        <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -1070,249 +1096,249 @@
       <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:7" ht="14.5">
-      <c r="A2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="9"/>
+      <c r="A2" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="16"/>
+      <c r="C2" s="17"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="24" t="s">
-        <v>32</v>
+      <c r="F2" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" ht="14.5">
-      <c r="A3" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
+      <c r="A3" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="16"/>
+      <c r="C3" s="17"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="24" t="s">
-        <v>33</v>
+      <c r="F3" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="G3" s="3"/>
     </row>
     <row r="4" spans="1:7" ht="14.5">
-      <c r="A4" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
+      <c r="A4" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="16"/>
+      <c r="C4" s="17"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="25" t="s">
-        <v>34</v>
+      <c r="F4" s="7" t="s">
+        <v>33</v>
       </c>
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" ht="14.5">
-      <c r="A5" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="12"/>
+      <c r="A5" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="19"/>
+      <c r="C5" s="20"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" ht="14.5">
+      <c r="A6" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" ht="14.5">
-      <c r="A6" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="15"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" ht="14.5">
+      <c r="A7" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" ht="14.5">
-      <c r="A7" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="18"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="26"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" spans="1:7" ht="14.5">
+      <c r="A8" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7" ht="14.5">
-      <c r="A8" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="20"/>
-      <c r="C8" s="21"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="29"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="25" t="s">
-        <v>35</v>
+      <c r="F8" s="7" t="s">
+        <v>34</v>
       </c>
       <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:7" ht="14.5">
-      <c r="A9" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="9"/>
+      <c r="A9" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="16"/>
+      <c r="C9" s="17"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" spans="1:7" ht="14.5">
+      <c r="A10" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" ht="14.5">
-      <c r="A10" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="21"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="23"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="25" t="s">
-        <v>36</v>
+      <c r="F10" s="7" t="s">
+        <v>35</v>
       </c>
       <c r="G10" s="3"/>
     </row>
     <row r="11" spans="1:7" ht="14.5">
-      <c r="A11" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="21"/>
+      <c r="A11" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="28"/>
+      <c r="C11" s="29"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
-      <c r="F11" s="22" t="s">
-        <v>37</v>
+      <c r="F11" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:7" ht="14.5">
-      <c r="A12" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="21"/>
+      <c r="A12" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="28"/>
+      <c r="C12" s="29"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
-      <c r="F12" s="24" t="s">
-        <v>38</v>
+      <c r="F12" s="6" t="s">
+        <v>37</v>
       </c>
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:7" ht="14.5">
-      <c r="A13" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="20"/>
-      <c r="C13" s="21"/>
+      <c r="A13" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="28"/>
+      <c r="C13" s="29"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="24" t="s">
-        <v>39</v>
+      <c r="F13" s="6" t="s">
+        <v>38</v>
       </c>
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="20"/>
-      <c r="C14" s="21"/>
+      <c r="A14" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="28"/>
+      <c r="C14" s="29"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:7" ht="14.5">
+      <c r="A15" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:7" ht="14.5">
-      <c r="A15" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="21"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="29"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="26" t="s">
-        <v>40</v>
+      <c r="F15" s="8" t="s">
+        <v>39</v>
       </c>
       <c r="G15" s="2"/>
     </row>
     <row r="16" spans="1:7" ht="14.5">
-      <c r="A16" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="9"/>
+      <c r="A16" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="31"/>
+      <c r="C16" s="32"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" spans="1:7" ht="14.5">
+      <c r="A17" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" ht="14.5">
-      <c r="A17" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="9"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="32"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
-      <c r="F17" s="25" t="s">
-        <v>41</v>
+      <c r="F17" s="7" t="s">
+        <v>40</v>
       </c>
       <c r="G17" s="2"/>
     </row>
     <row r="18" spans="1:7" ht="14.5">
-      <c r="A18" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="9"/>
+      <c r="A18" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="31"/>
+      <c r="C18" s="32"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G18" s="2"/>
+    </row>
+    <row r="19" spans="1:7" ht="14.5">
+      <c r="A19" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" ht="14.5">
-      <c r="A19" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="9"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="32"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" s="2"/>
+    </row>
+    <row r="20" spans="1:7" ht="14.5">
+      <c r="A20" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" spans="1:7" ht="14.5">
-      <c r="A20" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="9"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="32"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G20" s="2"/>
     </row>
@@ -1332,12 +1358,12 @@
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A6:C6"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>